<commit_message>
fix: align FQD workbook with 13 October release and procedure
Update the planned release date to 13-Oct-2026. Align readiness criterion G9 with Section 11.3, clarify controlled deliverable references in Appendix C, and remove obsolete procedure page numbers. Preserve formulas, validation, native tables and print settings.
</commit_message>
<xml_diff>
--- a/01-FQD/Appendices/PQD-FH_01_Universal_FQD_Templates.xlsx
+++ b/01-FQD/Appendices/PQD-FH_01_Universal_FQD_Templates.xlsx
@@ -2161,7 +2161,7 @@
         <v>Release date</v>
       </c>
       <c r="E8" s="7" t="d">
-        <v>2026-10-06T00:00:00.000Z</v>
+        <v>2026-10-13T00:00:00.000Z</v>
       </c>
       <c r="F8" s="1"/>
     </row>
@@ -2542,8 +2542,8 @@
       <c r="F38" s="1"/>
     </row>
     <row r="39" spans="1:6" ht="24.95" customHeight="1">
-      <c r="A39" s="25" t="s">
-        <v>60</v>
+      <c r="A39" s="25" t="str">
+        <v>Source: PQD-FH 01 Universal FQD Procedure, Rev. 1.00, Appendices A-I.</v>
       </c>
       <c r="B39" s="25"/>
       <c r="C39" s="25"/>
@@ -7553,12 +7553,12 @@
       <c r="F20" s="13"/>
       <c r="G20" s="17"/>
     </row>
-    <row r="21" spans="1:7" ht="48" customHeight="1">
+    <row r="21" spans="1:7" ht="90" customHeight="1">
       <c r="A21" s="9">
         <v>9</v>
       </c>
-      <c r="B21" s="9" t="s">
-        <v>266</v>
+      <c r="B21" s="9" t="str">
+        <v>Calibration / verification valid at the test date; any known subsequent equipment deficiencies assessed for impact on the results, with required actions completed or formally dispositioned against the applicable milestone criteria (Section 11.3)</v>
       </c>
       <c r="C21" s="13"/>
       <c r="D21" s="13"/>
@@ -13253,9 +13253,9 @@
       <c r="J7" s="30"/>
       <c r="K7" s="30"/>
     </row>
-    <row r="8" spans="1:11" ht="44.1" customHeight="1">
-      <c r="A8" s="25" t="s">
-        <v>111</v>
+    <row r="8" spans="1:11" ht="42" customHeight="1">
+      <c r="A8" s="25" t="str">
+        <v>One row per deliverable. Record its unique controlled reference and linked record IDs / revisions in Comment / N/A approval or a linked register (Section 7.2). Identify requirement revision and clause/activity. Record approved N/A dispositions.</v>
       </c>
       <c r="B8" s="25"/>
       <c r="C8" s="25"/>

</xml_diff>